<commit_message>
Tous les graphiques du portfolio faits dans Excel : 10 projets avec corrigé, exercice, tuto et CSV ; suppression des visualisations codées
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S2M5kbDHT3gJjWZ7gkW2je
</commit_message>
<xml_diff>
--- a/projets/nba-mi-distance/excel/nba-mi-distance-corrige.xlsx
+++ b/projets/nba-mi-distance/excel/nba-mi-distance-corrige.xlsx
@@ -23,6 +23,8 @@
     <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">'G1 Parts'!$A$1:$O$28</definedName>
     <definedName function="false" hidden="false" localSheetId="4" name="_xlnm.Print_Area" vbProcedure="false">'G2 Rendement'!$A$1:$O$28</definedName>
     <definedName function="false" hidden="false" localSheetId="7" name="_xlnm.Print_Area" vbProcedure="false">'G3 Correlation'!$A$1:$O$28</definedName>
+    <definedName function="false" hidden="false" localSheetId="8" name="_xlnm.Print_Area" vbProcedure="false">'Terrain 2004'!$A$1:$Z$20</definedName>
+    <definedName function="false" hidden="false" localSheetId="9" name="_xlnm.Print_Area" vbProcedure="false">'Terrain 2025'!$A$1:$Z$20</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -36,7 +38,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="75">
   <si>
-    <t xml:space="preserve">Le tir que la NBA a arrêté de financer — CORRIGÉ</t>
+    <t xml:space="preserve">Le tir que la NBA a arrêté de financer · CORRIGÉ</t>
   </si>
   <si>
     <t xml:space="preserve">Corrigé : toutes les formules sont en place, et chaque graphique a son onglet (G1 à G3). Ce sont ces graphiques qui sont sur le site.</t>
@@ -255,7 +257,7 @@
     <t xml:space="preserve">Carte des tirs 2003-04 : part des tirs (‰) par case de 2 × 2 pieds</t>
   </si>
   <si>
-    <t xml:space="preserve">Ligne du haut = au niveau du panier. Plus c'est rouge, plus on tire de là.</t>
+    <t xml:space="preserve">Ligne du haut = au niveau du panier. Plus c'est rouge, plus on tire de là. Même échelle de couleurs pour les deux saisons.</t>
   </si>
   <si>
     <t xml:space="preserve">Carte des tirs 2024-25 : part des tirs (‰) par case de 2 × 2 pieds</t>
@@ -1211,11 +1213,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="52749381"/>
-        <c:axId val="8221842"/>
+        <c:axId val="72713770"/>
+        <c:axId val="52135389"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="52749381"/>
+        <c:axId val="72713770"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1281,7 +1283,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="8221842"/>
+        <c:crossAx val="52135389"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1289,7 +1291,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="8221842"/>
+        <c:axId val="52135389"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="0.55"/>
@@ -1367,7 +1369,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="52749381"/>
+        <c:crossAx val="72713770"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1663,11 +1665,11 @@
         </c:ser>
         <c:gapWidth val="50"/>
         <c:overlap val="0"/>
-        <c:axId val="61423340"/>
-        <c:axId val="62599180"/>
+        <c:axId val="21997577"/>
+        <c:axId val="75114550"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="61423340"/>
+        <c:axId val="21997577"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -1699,7 +1701,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="62599180"/>
+        <c:crossAx val="75114550"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1707,7 +1709,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="62599180"/>
+        <c:axId val="75114550"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1783,7 +1785,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="61423340"/>
+        <c:crossAx val="21997577"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2208,11 +2210,11 @@
         </c:ser>
         <c:gapWidth val="40"/>
         <c:overlap val="0"/>
-        <c:axId val="1789461"/>
-        <c:axId val="17165070"/>
+        <c:axId val="66342550"/>
+        <c:axId val="30813992"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1789461"/>
+        <c:axId val="66342550"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2278,7 +2280,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="17165070"/>
+        <c:crossAx val="30813992"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2286,7 +2288,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="17165070"/>
+        <c:axId val="30813992"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2362,7 +2364,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1789461"/>
+        <c:crossAx val="66342550"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2749,7 +2751,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:Z20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -3986,7 +3988,7 @@
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="10"/>
-        <cfvo type="max" val="0"/>
+        <cfvo type="num" val="40"/>
         <color rgb="FFFFFFFF"/>
         <color rgb="FFF4B183"/>
         <color rgb="FFC0392B"/>
@@ -3994,8 +3996,8 @@
     </cfRule>
   </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.2" right="0.2" top="0.2" bottom="0.2" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -5927,7 +5929,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:Z20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -7180,7 +7182,7 @@
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="10"/>
-        <cfvo type="max" val="0"/>
+        <cfvo type="num" val="40"/>
         <color rgb="FFFFFFFF"/>
         <color rgb="FFF4B183"/>
         <color rgb="FFC0392B"/>
@@ -7188,8 +7190,8 @@
     </cfRule>
   </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.2" right="0.2" top="0.2" bottom="0.2" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>